<commit_message>
AB2D-7308 v3 data dictionary followup (#200)
Followup to #196
</commit_message>
<xml_diff>
--- a/src/assets/downloads/ab2d-v3-data-dictionary-migration.xlsx
+++ b/src/assets/downloads/ab2d-v3-data-dictionary-migration.xlsx
@@ -16,202 +16,6 @@
     <pivotCache cacheId="0" r:id="rId9"/>
   </pivotCaches>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
-  <authors>
-    <author>tc={6f060db2-eff1-4c73-8641-98341795462c}</author>
-    <author>tc={8d71795f-db08-47ab-a83c-e2a499cdebb6}</author>
-  </authors>
-  <commentList>
-    <comment authorId="0" xr:uid="{6f060db2-eff1-4c73-8641-98341795462c}" ref="A1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Remove "No change"
-</t>
-      </text>
-    </comment>
-    <comment authorId="1" xr:uid="{8d71795f-db08-47ab-a83c-e2a499cdebb6}" ref="A1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	List element names under each category
-Reply:
-	Do we need to @andrew.harnish1@cms.hhs.gov ? the filter on the sheet should give them that list . If you prefer to add still, I can. Let me know
-Reply:
-	I really like how the old one was formatted. If you create this table as a pivot table its as easy as adding one more data element into the table
-Reply:
-	Done
-Reply:
-	Marked as resolved
-Reply:
-	Re-opened
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
-  <authors>
-    <author>tc={100087d1-04c6-4edc-8e60-3897b2f8a40e}</author>
-  </authors>
-  <commentList>
-    <comment authorId="0" xr:uid="{100087d1-04c6-4edc-8e60-3897b2f8a40e}" ref="B2">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	AB2D instead of BCDA?
-Reply:
-	also, new link to the BB IG https://build.fhir.org/ig/HL7/carin-bb/
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
-  <authors>
-    <author>tc={0688e772-6e18-4964-a1e6-87a29ec9a5dd}</author>
-    <author>tc={47515430-a677-413a-839f-8d4e25eccda0}</author>
-    <author>tc={51b3fb9b-255e-4173-a2d8-af34c78ac995}</author>
-    <author>tc={51fcca03-7a55-4085-a830-a00695e762a8}</author>
-    <author>tc={67ed361c-ce1b-4ef1-b85f-4f4937a99bfe}</author>
-    <author>tc={680c05fc-8535-46c9-9547-0d1204ac1112}</author>
-    <author>tc={7e0fbbac-1a18-4424-9883-08bc0f5dad0f}</author>
-    <author>tc={a698efde-c5fe-412d-81e0-792ab0fb0de3}</author>
-    <author>tc={a8d90c21-0e8b-4588-bcef-f44de978ecfb}</author>
-    <author>tc={b030fdc2-1191-40d1-9f30-da30b07724a6}</author>
-    <author>tc={d2b22c25-565f-4dd7-a254-f1aa8dda2464}</author>
-  </authors>
-  <commentList>
-    <comment authorId="0" xr:uid="{0688e772-6e18-4964-a1e6-87a29ec9a5dd}" ref="J1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Add "v1-" to column title
-</t>
-      </text>
-    </comment>
-    <comment authorId="1" xr:uid="{47515430-a677-413a-839f-8d4e25eccda0}" ref="R29">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	this actually existed in v2. there were a couple extensions that represented the claim control number
-Reply:
-	Changed it as "New StructureDefinition/CodeSystem URL"
-</t>
-      </text>
-    </comment>
-    <comment authorId="2" xr:uid="{51b3fb9b-255e-4173-a2d8-af34c78ac995}" ref="R1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	v3-R4 discriminator?
-Reply:
-	BFD combined FHIR element and Discriminator from v2 into a valid FHIRPath in v3. So it doesn't make sense to add discriminator for v3
-Reply:
-	Is there anything of value to share with the v3 FHIRPath that supplements discriminator info?
-</t>
-      </text>
-    </comment>
-    <comment authorId="3" xr:uid="{51fcca03-7a55-4085-a830-a00695e762a8}" ref="L1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	v2-R4 discriminator?
-Reply:
-	We should figure out how to indicate that this is a old element and potentially note it will be deprecated
-Reply:
-	Marked as resolved
-Reply:
-	v2-R4 discriminator column was hidden, so now its part of the sheet.
-Re-opened
-</t>
-      </text>
-    </comment>
-    <comment authorId="4" xr:uid="{67ed361c-ce1b-4ef1-b85f-4f4937a99bfe}" ref="T1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Need to add definition of "breaking change" to "definitions" or "glossary" tab
-</t>
-      </text>
-    </comment>
-    <comment authorId="5" xr:uid="{680c05fc-8535-46c9-9547-0d1204ac1112}" ref="K1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Can we remove?
-</t>
-      </text>
-    </comment>
-    <comment authorId="6" xr:uid="{7e0fbbac-1a18-4424-9883-08bc0f5dad0f}" ref="K1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	add "v1-" to column title
-</t>
-      </text>
-    </comment>
-    <comment authorId="7" xr:uid="{a698efde-c5fe-412d-81e0-792ab0fb0de3}" ref="U1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Need to add definition of effort rating to "definitions" or "glossary" tab
-Reply:
-	Consider removing. Can be relative. Our Low might be another's Medium or High
-</t>
-      </text>
-    </comment>
-    <comment authorId="8" xr:uid="{a8d90c21-0e8b-4588-bcef-f44de978ecfb}" ref="R59">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	ope, this is actually still in v3, but in a different spot. It is in ExplanationOfBenefit.meta.tag.where(system='https://bluebutton.cms.gov/fhir/CodeSystem/Final-Action').code
-Reply:
-	Good catch Colby, missed it
-</t>
-      </text>
-    </comment>
-    <comment authorId="9" xr:uid="{b030fdc2-1191-40d1-9f30-da30b07724a6}" ref="G1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	We should figure out how to indicate that this is a old element and potentially note it will be deprecated
-</t>
-      </text>
-    </comment>
-    <comment authorId="10" xr:uid="{d2b22c25-565f-4dd7-a254-f1aa8dda2464}" ref="I1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Add "v1-" to column title
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4228,18 +4032,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
-<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
-</file>
-
-<file path=xl/documenttasks/documenttask2.xml><?xml version="1.0" encoding="utf-8"?>
-<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
-</file>
-
-<file path=xl/documenttasks/documenttask3.xml><?xml version="1.0" encoding="utf-8"?>
-<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -4257,14 +4049,7 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Anonymous" id="{1ed149f1-c230-4583-b173-845464fcaf7d}" providerId="google-sheets"/>
-  <x18tc:person displayName="Natalie Watkins" id="{d5ff3ef0-47a0-4370-8648-915aae88d725}" providerId="google-sheets"/>
-  <x18tc:person displayName="Sravanti Adibhatla" id="{8ba88ff1-9cd0-4f59-9755-ac7961817118}" providerId="google-sheets"/>
-  <x18tc:person displayName="Andrew Harnish" id="{317e8d9b-b4c7-486c-9ddb-6939b56fc42e}" providerId="google-sheets"/>
-  <x18tc:person displayName="Colby Seyferth" id="{d6353024-ee04-4541-9651-ae880766fab2}" providerId="google-sheets"/>
-  <x18tc:person displayName="andrew.harnish1@cms.hhs.gov" id="{465d6a29-5344-45ed-83db-6d3333c8024e}" userId="andrew.harnish1@cms.hhs.gov" providerId="google-sheets"/>
-</x18tc:personList>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7084,121 +6869,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A1" dT="2026-02-17T18:41:30.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{6f060db2-eff1-4c73-8641-98341795462c}" done="1">
-    <x18tc:text xml:space="preserve">Remove "No change"</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-02-17T18:41:47.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{8d71795f-db08-47ab-a83c-e2a499cdebb6}" done="1">
-    <x18tc:text xml:space="preserve">List element names under each category</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-02-18T22:50:47.00" personId="{8ba88ff1-9cd0-4f59-9755-ac7961817118}" id="{ee47783c-322b-459a-8e12-a4a9a0bc1a3b}" parentId="{8d71795f-db08-47ab-a83c-e2a499cdebb6}">
-    <x18tc:text xml:space="preserve">Do we need to @andrew.harnish1@cms.hhs.gov ? the filter on the sheet should give them that list . If you prefer to add still, I can. Let me know</x18tc:text>
-    <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{465d6a29-5344-45ed-83db-6d3333c8024e}" mentionId="{ac7368f7-8c0d-4efe-a268-59cbd637ca1a}" startIndex="14" length="28"/>
-    </x18tc:mentions>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-02-19T18:13:43.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{ae51431d-1574-49ee-ae0a-70f052f34588}" parentId="{8d71795f-db08-47ab-a83c-e2a499cdebb6}">
-    <x18tc:text xml:space="preserve">I really like how the old one was formatted. If you create this table as a pivot table its as easy as adding one more data element into the table</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-02-19T18:56:41.00" personId="{317e8d9b-b4c7-486c-9ddb-6939b56fc42e}" id="{c7299e75-20be-410a-91b2-b70651b6fe14}" parentId="{8d71795f-db08-47ab-a83c-e2a499cdebb6}">
-    <x18tc:text xml:space="preserve">Done</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-02-19T18:56:53.00" personId="{317e8d9b-b4c7-486c-9ddb-6939b56fc42e}" id="{6c0b9cfe-855d-4131-ab24-92839b4a8037}" parentId="{8d71795f-db08-47ab-a83c-e2a499cdebb6}">
-    <x18tc:text xml:space="preserve">Marked as resolved</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-02-19T18:57:29.00" personId="{317e8d9b-b4c7-486c-9ddb-6939b56fc42e}" id="{4e0ed600-9d65-489c-90ed-cfd62dbd12ef}" parentId="{8d71795f-db08-47ab-a83c-e2a499cdebb6}">
-    <x18tc:text xml:space="preserve">Re-opened</x18tc:text>
-  </x18tc:threadedComment>
-</x18tc:ThreadedComments>
-</file>
-
-<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B2" dT="2026-02-17T19:20:56.00" personId="{d5ff3ef0-47a0-4370-8648-915aae88d725}" id="{100087d1-04c6-4edc-8e60-3897b2f8a40e}" done="1">
-    <x18tc:text xml:space="preserve">AB2D instead of BCDA?</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="B2" dT="2026-02-17T19:22:17.00" personId="{d5ff3ef0-47a0-4370-8648-915aae88d725}" id="{bfbcedc3-a4d5-4995-8b9d-dc8a22696cfd}" parentId="{100087d1-04c6-4edc-8e60-3897b2f8a40e}">
-    <x18tc:text xml:space="preserve">also, new link to the BB IG https://build.fhir.org/ig/HL7/carin-bb/</x18tc:text>
-    <x18tc:extLst>
-      <ext uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
-        <xltc2:checksum/>
-        <xltc2:hyperlink startIndex="28" length="39" url="https://build.fhir.org/ig/HL7/carin-bb/"/>
-      </ext>
-    </x18tc:extLst>
-  </x18tc:threadedComment>
-</x18tc:ThreadedComments>
-</file>
-
-<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="R29" dT="2026-04-27T18:14:31.00" personId="{d6353024-ee04-4541-9651-ae880766fab2}" id="{47515430-a677-413a-839f-8d4e25eccda0}" done="0">
-    <x18tc:text xml:space="preserve">this actually existed in v2. there were a couple extensions that represented the claim control number</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="R29" dT="2026-04-27T19:08:48.00" personId="{8ba88ff1-9cd0-4f59-9755-ac7961817118}" id="{4a68508d-14ea-4d5e-83a8-6fddc8519ce9}" parentId="{47515430-a677-413a-839f-8d4e25eccda0}">
-    <x18tc:text xml:space="preserve">Changed it as "New StructureDefinition/CodeSystem URL"</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K1" dT="2026-02-17T18:37:33.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{7e0fbbac-1a18-4424-9883-08bc0f5dad0f}" done="1">
-    <x18tc:text xml:space="preserve">add "v1-" to column title</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="R59" dT="2026-04-20T16:56:55.00" personId="{d6353024-ee04-4541-9651-ae880766fab2}" id="{a8d90c21-0e8b-4588-bcef-f44de978ecfb}" done="1">
-    <x18tc:text xml:space="preserve">ope, this is actually still in v3, but in a different spot. It is in ExplanationOfBenefit.meta.tag.where(system='https://bluebutton.cms.gov/fhir/CodeSystem/Final-Action').code</x18tc:text>
-    <x18tc:extLst>
-      <ext uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
-        <xltc2:checksum/>
-        <xltc2:hyperlink startIndex="113" length="62" url="https://bluebutton.cms.gov/fhir/CodeSystem/Final-Action').code"/>
-      </ext>
-    </x18tc:extLst>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="R59" dT="2026-04-20T17:25:50.00" personId="{8ba88ff1-9cd0-4f59-9755-ac7961817118}" id="{66062ec2-5116-4be7-b37a-10e457b6fcf6}" parentId="{a8d90c21-0e8b-4588-bcef-f44de978ecfb}">
-    <x18tc:text xml:space="preserve">Good catch Colby, missed it</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="J1" dT="2026-02-17T18:37:55.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{0688e772-6e18-4964-a1e6-87a29ec9a5dd}" done="1">
-    <x18tc:text xml:space="preserve">Add "v1-" to column title</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I1" dT="2026-02-17T18:38:14.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{d2b22c25-565f-4dd7-a254-f1aa8dda2464}" done="1">
-    <x18tc:text xml:space="preserve">Add "v1-" to column title</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="T1" dT="2026-02-17T18:40:06.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{67ed361c-ce1b-4ef1-b85f-4f4937a99bfe}" done="0">
-    <x18tc:text xml:space="preserve">Need to add definition of "breaking change" to "definitions" or "glossary" tab</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L1" dT="2026-02-17T18:34:51.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{51fcca03-7a55-4085-a830-a00695e762a8}" done="0">
-    <x18tc:text xml:space="preserve">v2-R4 discriminator?</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L1" dT="2026-02-17T18:36:54.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{53f399c9-892b-4d0d-b4d9-9efb12c66ad0}" parentId="{51fcca03-7a55-4085-a830-a00695e762a8}">
-    <x18tc:text xml:space="preserve">We should figure out how to indicate that this is a old element and potentially note it will be deprecated</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L1" dT="2026-02-18T22:47:01.00" personId="{8ba88ff1-9cd0-4f59-9755-ac7961817118}" id="{3d88da56-3577-46e8-9567-45e968db420c}" parentId="{51fcca03-7a55-4085-a830-a00695e762a8}">
-    <x18tc:text xml:space="preserve">Marked as resolved</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L1" dT="2026-02-18T22:49:28.00" personId="{8ba88ff1-9cd0-4f59-9755-ac7961817118}" id="{0d3833fd-9b8c-4cae-99df-d71fdf2b1e1b}" parentId="{51fcca03-7a55-4085-a830-a00695e762a8}">
-    <x18tc:text xml:space="preserve">v2-R4 discriminator column was hidden, so now its part of the sheet.
-Re-opened</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="U1" dT="2026-02-17T18:40:46.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{a698efde-c5fe-412d-81e0-792ab0fb0de3}" done="0">
-    <x18tc:text xml:space="preserve">Need to add definition of effort rating to "definitions" or "glossary" tab</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="U1" dT="2026-02-19T19:07:19.00" personId="{317e8d9b-b4c7-486c-9ddb-6939b56fc42e}" id="{d18e35fe-dc48-4e8f-898a-b2d6c1d23b13}" parentId="{a698efde-c5fe-412d-81e0-792ab0fb0de3}">
-    <x18tc:text xml:space="preserve">Consider removing. Can be relative. Our Low might be another's Medium or High</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="R1" dT="2026-02-17T18:35:05.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{51b3fb9b-255e-4173-a2d8-af34c78ac995}" done="0">
-    <x18tc:text xml:space="preserve">v3-R4 discriminator?</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="R1" dT="2026-02-18T22:47:42.00" personId="{8ba88ff1-9cd0-4f59-9755-ac7961817118}" id="{6acc6e50-ab8d-4d60-880b-d2c556c7fe50}" parentId="{51b3fb9b-255e-4173-a2d8-af34c78ac995}">
-    <x18tc:text xml:space="preserve">BFD combined FHIR element and Discriminator from v2 into a valid FHIRPath in v3. So it doesn't make sense to add discriminator for v3</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="R1" dT="2026-02-19T18:54:44.00" personId="{317e8d9b-b4c7-486c-9ddb-6939b56fc42e}" id="{8317a97b-f7e7-415b-bf88-6e085bdcda30}" parentId="{51b3fb9b-255e-4173-a2d8-af34c78ac995}">
-    <x18tc:text xml:space="preserve">Is there anything of value to share with the v3 FHIRPath that supplements discriminator info?</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="G1" dT="2026-02-17T18:36:38.00" personId="{1ed149f1-c230-4583-b173-845464fcaf7d}" id="{b030fdc2-1191-40d1-9f30-da30b07724a6}" done="0">
-    <x18tc:text xml:space="preserve">We should figure out how to indicate that this is a old element and potentially note it will be deprecated</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K1" dT="2026-02-19T19:10:22.00" personId="{317e8d9b-b4c7-486c-9ddb-6939b56fc42e}" id="{680c05fc-8535-46c9-9547-0d1204ac1112}" done="0">
-    <x18tc:text xml:space="preserve">Can we remove?</x18tc:text>
-  </x18tc:threadedComment>
-</x18tc:ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
@@ -7336,10 +7006,9 @@
       <c r="C14" s="6"/>
     </row>
   </sheetData>
-  <drawing r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7410,10 +7079,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <drawing r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -23824,14 +23492,13 @@
   </sheetData>
   <autoFilter ref="$A$1:$U$253"/>
   <hyperlinks>
-    <hyperlink r:id="rId4" ref="W28"/>
-    <hyperlink r:id="rId5" ref="R29"/>
-    <hyperlink r:id="rId6" ref="R247"/>
+    <hyperlink r:id="rId1" ref="W28"/>
+    <hyperlink r:id="rId2" ref="R29"/>
+    <hyperlink r:id="rId3" ref="R247"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId7"/>
-  <legacyDrawing r:id="rId8"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>